<commit_message>
Tested OpenCode with Unit Generation Skills
</commit_message>
<xml_diff>
--- a/project1/reports/opencode/comparison prompt 1.xlsx
+++ b/project1/reports/opencode/comparison prompt 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Project Bachelor\project 1 small\reports\opencode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861B013B-156A-4D5B-A7F5-4DCEAD938A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB456CF6-797F-4D16-9867-0DAB498BED6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="7" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
   </bookViews>
   <sheets>
     <sheet name="MyMath.checkSign(int)" sheetId="1" r:id="rId1"/>
@@ -2842,8 +2842,8 @@
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>11</v>
+      <c r="D4" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>

</xml_diff>